<commit_message>
corretto linee verticali dei grafici
</commit_message>
<xml_diff>
--- a/MISURE-MALFUNZ.-MANUTENZ. PEN3.xlsx
+++ b/MISURE-MALFUNZ.-MANUTENZ. PEN3.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="111">
   <si>
     <t xml:space="preserve">data inizio misure</t>
   </si>
@@ -37,6 +37,9 @@
     <t xml:space="preserve">riavvio</t>
   </si>
   <si>
+    <t xml:space="preserve">Casa Simoncelli</t>
+  </si>
+  <si>
     <t xml:space="preserve">N.B. Il 30/07/2020 ore 15:35 è stato staccato il PEN3 di PCA Tech. e alle ore 15:52 è stato avviato il PEN3 comunale appena revisionato.</t>
   </si>
   <si>
@@ -134,9 +137,6 @@
   </si>
   <si>
     <t xml:space="preserve">ago</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Casa Simoncelli</t>
   </si>
   <si>
     <t xml:space="preserve">Il 4 febbraio alle 15:00 hanno tolto la corrente per tagliare l'erba e l'hanno rimessa solo l'8 febbraio alle 14:40 (la rilevazione vento è ripartita da sola, mentre il pen3 l'ho fatto ripartire io)</t>
@@ -824,11 +824,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1645,13 +1645,23 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7"/>
+      <c r="A16" s="7" t="s">
+        <v>4</v>
+      </c>
       <c r="B16" s="11"/>
       <c r="C16" s="12"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="18"/>
+      <c r="D16" s="17" t="n">
+        <v>42958</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>0.618055555555556</v>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>42959</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>0.310416666666667</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2"/>
@@ -1768,13 +1778,23 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7"/>
+      <c r="A29" s="7" t="s">
+        <v>4</v>
+      </c>
       <c r="B29" s="11"/>
       <c r="C29" s="12"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="18"/>
+      <c r="D29" s="17" t="n">
+        <v>43322</v>
+      </c>
+      <c r="E29" s="18" t="n">
+        <v>0.449305555555556</v>
+      </c>
+      <c r="F29" s="17" t="n">
+        <v>43322</v>
+      </c>
+      <c r="G29" s="18" t="n">
+        <v>0.541666666666667</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2"/>
@@ -2137,7 +2157,7 @@
     </row>
     <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="31" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B74" s="32"/>
       <c r="C74" s="32"/>
@@ -2150,7 +2170,7 @@
     </row>
     <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="31" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B75" s="20"/>
       <c r="C75" s="33"/>
@@ -2163,7 +2183,7 @@
     </row>
     <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="31" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B76" s="20"/>
       <c r="C76" s="33"/>
@@ -2187,24 +2207,24 @@
     <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B80" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C80" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D80" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E80" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2226,7 +2246,7 @@
     </row>
     <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B82" s="40"/>
       <c r="C82" s="40"/>
@@ -2235,19 +2255,19 @@
     </row>
     <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B83" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C83" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D83" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E83" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2270,7 +2290,7 @@
     </row>
     <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B85" s="40"/>
       <c r="C85" s="40"/>
@@ -2280,19 +2300,19 @@
     </row>
     <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B86" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C86" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D86" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E86" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J86" s="29"/>
     </row>
@@ -2316,7 +2336,7 @@
     </row>
     <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B88" s="40"/>
       <c r="C88" s="40"/>
@@ -2326,19 +2346,19 @@
     </row>
     <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B89" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C89" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D89" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E89" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2492,7 +2512,7 @@
     <row r="106" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="107" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B107" s="29" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J107" s="20"/>
       <c r="K107" s="20"/>
@@ -2507,14 +2527,14 @@
     </row>
     <row r="109" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="31" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B109" s="32"/>
       <c r="C109" s="32"/>
     </row>
     <row r="110" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="31" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B110" s="32"/>
       <c r="C110" s="32"/>
@@ -2527,7 +2547,7 @@
     </row>
     <row r="111" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="31" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B111" s="32"/>
       <c r="C111" s="32"/>
@@ -2540,7 +2560,7 @@
     </row>
     <row r="112" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B112" s="32"/>
       <c r="C112" s="32"/>
@@ -2553,7 +2573,7 @@
     </row>
     <row r="113" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="46" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B113" s="47"/>
       <c r="C113" s="47"/>
@@ -2562,36 +2582,36 @@
     <row r="115" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="116" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G116" s="29" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B117" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C117" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D117" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E117" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G117" s="37" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H117" s="37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I117" s="37" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2623,7 +2643,7 @@
     </row>
     <row r="119" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B119" s="40"/>
       <c r="C119" s="40"/>
@@ -2635,28 +2655,28 @@
     </row>
     <row r="120" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B120" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C120" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D120" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E120" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G120" s="37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H120" s="37" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I120" s="37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2696,7 +2716,7 @@
     </row>
     <row r="122" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B122" s="40"/>
       <c r="C122" s="40"/>
@@ -2716,28 +2736,28 @@
     </row>
     <row r="123" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B123" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C123" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D123" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E123" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G123" s="37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H123" s="37" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I123" s="37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J123" s="31"/>
       <c r="K123" s="31"/>
@@ -2777,7 +2797,7 @@
     </row>
     <row r="125" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="12" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B125" s="40"/>
       <c r="C125" s="40"/>
@@ -2786,19 +2806,19 @@
     </row>
     <row r="126" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B126" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C126" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D126" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E126" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="127" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2859,7 +2879,7 @@
       <c r="J131" s="7"/>
       <c r="K131" s="7"/>
       <c r="L131" s="37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M131" s="7"/>
       <c r="N131" s="7"/>
@@ -2898,7 +2918,7 @@
     </row>
     <row r="133" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B133" s="7"/>
       <c r="C133" s="7"/>
@@ -2925,7 +2945,7 @@
     </row>
     <row r="134" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B134" s="7"/>
       <c r="C134" s="7"/>
@@ -2951,7 +2971,7 @@
     </row>
     <row r="135" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B135" s="7"/>
       <c r="C135" s="7"/>
@@ -2977,7 +2997,7 @@
     </row>
     <row r="136" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B136" s="7"/>
       <c r="C136" s="7"/>
@@ -2999,7 +3019,7 @@
     </row>
     <row r="137" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B137" s="7"/>
       <c r="C137" s="7"/>
@@ -3021,7 +3041,7 @@
     </row>
     <row r="138" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B138" s="7"/>
       <c r="C138" s="7"/>
@@ -3040,7 +3060,7 @@
     </row>
     <row r="139" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B139" s="7"/>
       <c r="C139" s="7"/>
@@ -3062,7 +3082,7 @@
     </row>
     <row r="140" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B140" s="7"/>
       <c r="C140" s="7"/>
@@ -3099,28 +3119,28 @@
     </row>
     <row r="145" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B145" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C145" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D145" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E145" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G145" s="37" t="s">
         <v>44</v>
       </c>
       <c r="H145" s="37" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I145" s="37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3168,19 +3188,19 @@
     </row>
     <row r="148" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B148" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C148" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D148" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E148" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G148" s="39"/>
       <c r="H148" s="39" t="n">
@@ -3234,28 +3254,28 @@
     </row>
     <row r="151" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B151" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C151" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D151" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E151" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G151" s="37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H151" s="37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I151" s="37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3317,13 +3337,13 @@
     </row>
     <row r="156" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="J156" s="37" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K156" s="37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L156" s="37" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="157" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3391,7 +3411,7 @@
     </row>
     <row r="161" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B161" s="7"/>
       <c r="C161" s="7"/>
@@ -3416,7 +3436,7 @@
     </row>
     <row r="162" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B162" s="7"/>
       <c r="C162" s="7"/>
@@ -3436,10 +3456,10 @@
         <v>47</v>
       </c>
       <c r="J162" s="37" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K162" s="37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L162" s="37" t="s">
         <v>39</v>
@@ -3447,7 +3467,7 @@
     </row>
     <row r="163" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B163" s="7"/>
       <c r="C163" s="7"/>
@@ -3478,7 +3498,7 @@
     </row>
     <row r="164" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B164" s="7"/>
       <c r="C164" s="7"/>
@@ -3505,7 +3525,7 @@
     </row>
     <row r="165" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B165" s="7"/>
       <c r="C165" s="7"/>
@@ -3530,7 +3550,7 @@
     </row>
     <row r="166" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B166" s="7"/>
       <c r="C166" s="7"/>
@@ -3553,7 +3573,7 @@
     </row>
     <row r="167" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B167" s="7"/>
       <c r="C167" s="7"/>
@@ -3564,7 +3584,7 @@
     </row>
     <row r="168" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B168" s="7"/>
       <c r="C168" s="7"/>
@@ -3612,28 +3632,28 @@
     </row>
     <row r="177" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B177" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C177" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D177" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E177" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G177" s="37" t="s">
         <v>44</v>
       </c>
       <c r="H177" s="37" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I177" s="37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3681,19 +3701,19 @@
     </row>
     <row r="180" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B180" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C180" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D180" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E180" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G180" s="39"/>
       <c r="H180" s="39" t="n">
@@ -3746,28 +3766,28 @@
     </row>
     <row r="183" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="36" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B183" s="37" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C183" s="37" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D183" s="37" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E183" s="37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G183" s="37" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H183" s="37" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I183" s="37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3816,13 +3836,13 @@
     </row>
     <row r="188" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="J188" s="37" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K188" s="37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L188" s="37" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3884,7 +3904,7 @@
     </row>
     <row r="193" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B193" s="7"/>
       <c r="C193" s="7"/>
@@ -3909,7 +3929,7 @@
     </row>
     <row r="194" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B194" s="7"/>
       <c r="C194" s="7"/>
@@ -3929,10 +3949,10 @@
         <v>52</v>
       </c>
       <c r="J194" s="37" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K194" s="37" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L194" s="37" t="s">
         <v>39</v>
@@ -3940,7 +3960,7 @@
     </row>
     <row r="195" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B195" s="7"/>
       <c r="C195" s="7"/>
@@ -3971,7 +3991,7 @@
     </row>
     <row r="196" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B196" s="7"/>
       <c r="C196" s="7"/>
@@ -3996,7 +4016,7 @@
     </row>
     <row r="197" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B197" s="7"/>
       <c r="C197" s="7"/>
@@ -4010,7 +4030,7 @@
     </row>
     <row r="198" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B198" s="7"/>
       <c r="C198" s="7"/>
@@ -4024,7 +4044,7 @@
     </row>
     <row r="199" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B199" s="7"/>
       <c r="C199" s="7"/>
@@ -4035,7 +4055,7 @@
     </row>
     <row r="200" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="7" t="s">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="B200" s="7"/>
       <c r="C200" s="7"/>

</xml_diff>